<commit_message>
Update BOM with chassis, wiring and distribution selections
</commit_message>
<xml_diff>
--- a/Documentation/BOM/SentinelT_Bill_of_Materials.xlsx
+++ b/Documentation/BOM/SentinelT_Bill_of_Materials.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="R9367dcbaae5e4fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Submission_Checklist" sheetId="2" r:id="R995a0a3f78ed4f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="R88e8c55008944177"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Submission_Checklist" sheetId="2" r:id="R4169c6a370e746be"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -256,14 +256,14 @@
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -517,7 +517,7 @@
         <x:v>&lt; 5.000 kg</x:v>
       </x:c>
       <x:c r="I2" t="str">
-        <x:v>PARTIAL PROCUREMENT DATA</x:v>
+        <x:v>NEAR-COMPLETE PROCUREMENT DATA</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -551,58 +551,62 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="20" t="str">
-        <x:v>Chassis material / base plate</x:v>
+        <x:v>HDPE sheet 6mm — chassis/base and shared armor stock</x:v>
       </x:c>
       <x:c r="B5" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C5" s="22"/>
+      <x:c r="C5" s="22" t="n">
+        <x:v>1943.5</x:v>
+      </x:c>
       <x:c r="D5" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Plastic World</x:v>
       </x:c>
       <x:c r="E5" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>HDPNAT06,0X20001000</x:v>
       </x:c>
       <x:c r="F5" s="20" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="G5" s="22" t="str">
+        <x:v>https://plasticworld.co.za/shop/hdpe-sheet-6mm/</x:v>
+      </x:c>
+      <x:c r="G5" s="22" t="n">
         <x:f>IF(ISNUMBER(C5),B5*C5,"TBD")</x:f>
-        <x:v>TBD</x:v>
+        <x:v>1943.5</x:v>
       </x:c>
       <x:c r="H5" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="I5" s="20" t="str">
-        <x:v>Final material/thickness to be selected</x:v>
+        <x:v>2m x 1m x 6mm HDPE sheet. Only the required cut sections are used in the robot; full-sheet purchase mass is not robot mass.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="str">
-        <x:v>Structural / armor material</x:v>
+        <x:v>Structural / armor panels cut from chassis HDPE stock</x:v>
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C6" s="22"/>
+      <x:c r="C6" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="D6" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Plastic World</x:v>
       </x:c>
       <x:c r="E6" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Shared stock: HDPNAT06,0X20001000</x:v>
       </x:c>
       <x:c r="F6" s="20" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="G6" s="22" t="str">
+        <x:v>https://plasticworld.co.za/shop/hdpe-sheet-6mm/</x:v>
+      </x:c>
+      <x:c r="G6" s="22" t="n">
         <x:f>IF(ISNUMBER(C6),B6*C6,"TBD")</x:f>
-        <x:v>TBD</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="I6" s="20" t="str">
-        <x:v>Outer armor and guards</x:v>
+        <x:v>Armor panels are cut from the same 6mm HDPE sheet purchased on row 5, so no duplicate material cost is charged.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -877,30 +881,32 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="20" t="str">
-        <x:v>Power distribution / terminal block</x:v>
+        <x:v>Power distribution terminal block — 100A 4-way</x:v>
       </x:c>
       <x:c r="B16" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C16" s="22"/>
+      <x:c r="C16" s="22" t="n">
+        <x:v>179</x:v>
+      </x:c>
       <x:c r="D16" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>GeeWiz</x:v>
       </x:c>
       <x:c r="E16" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>AC-TB-1004</x:v>
       </x:c>
       <x:c r="F16" s="20" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="G16" s="22" t="str">
+        <x:v>https://www.geewiz.co.za/wiring-accessories/670146-terminal-block-100a-4-way.html</x:v>
+      </x:c>
+      <x:c r="G16" s="22" t="n">
         <x:f>IF(ISNUMBER(C16),B16*C16,"TBD")</x:f>
-        <x:v>TBD</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="H16" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="I16" s="20" t="str">
-        <x:v>Distributes battery power to subsystems</x:v>
+        <x:v>100A 4-way terminal block for compact battery-power distribution. Final branch protection and enclosure layout must be verified.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -935,114 +941,122 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="20" t="str">
-        <x:v>Electrical wiring set</x:v>
+        <x:v>10mm² silicone power-wire set (2m red + 2m black)</x:v>
       </x:c>
       <x:c r="B18" s="20" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C18" s="22"/>
+      <x:c r="C18" s="22" t="n">
+        <x:v>334</x:v>
+      </x:c>
       <x:c r="D18" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>GeeWiz</x:v>
       </x:c>
       <x:c r="E18" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>352M0047 / 352M0277</x:v>
       </x:c>
       <x:c r="F18" s="20" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="G18" s="22" t="str">
+        <x:v>https://www.geewiz.co.za/cables-adapters/590608-silicone-wire-m-s-csa100-o66-red-debulk-800464pm.html</x:v>
+      </x:c>
+      <x:c r="G18" s="22" t="n">
         <x:f>IF(ISNUMBER(C18),B18*C18,"TBD")</x:f>
-        <x:v>TBD</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="H18" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="I18" s="20" t="str">
-        <x:v>Wire gauge to be selected from current requirements</x:v>
+        <x:v>2m red + 2m black flexible silicone wire. Supplier lists 10mm² conductors at 112A; black companion item is 352M0277.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="20" t="str">
-        <x:v>Bearings</x:v>
+        <x:v>Drive-shaft support bearings</x:v>
       </x:c>
       <x:c r="B19" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C19" s="22"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C19" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="D19" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Not required for selected direct-drive wheel system</x:v>
       </x:c>
       <x:c r="E19" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="F19" s="20" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="G19" s="22" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="G19" s="22" t="n">
         <x:f>IF(ISNUMBER(C19),B19*C19,"TBD")</x:f>
-        <x:v>TBD</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H19" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="I19" s="20" t="str">
-        <x:v>Quantity/spec depends on final mechanical assembly</x:v>
+        <x:v>Selected wheels mount directly to the 6mm gearmotor shafts, so separate wheel-support bearings are not required for the current drivetrain.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="20" t="str">
-        <x:v>Shafts / axles</x:v>
+        <x:v>Separate drive shafts / axles</x:v>
       </x:c>
       <x:c r="B20" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C20" s="22"/>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C20" s="22" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="D20" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Not required for selected direct-drive wheel system</x:v>
       </x:c>
       <x:c r="E20" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>N/A</x:v>
       </x:c>
       <x:c r="F20" s="20" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="G20" s="22" t="str">
+        <x:v>N/A</x:v>
+      </x:c>
+      <x:c r="G20" s="22" t="n">
         <x:f>IF(ISNUMBER(C20),B20*C20,"TBD")</x:f>
-        <x:v>TBD</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H20" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Verified</x:v>
       </x:c>
       <x:c r="I20" s="20" t="str">
-        <x:v>Diameter/material TBD</x:v>
+        <x:v>Selected 37D gearmotors provide the 6mm output shafts used by the wheels; no separate drive axles are required.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="20" t="str">
-        <x:v>Fasteners and spacers</x:v>
+        <x:v>M4 stainless fastener sets (bolt + nut)</x:v>
       </x:c>
       <x:c r="B21" s="20" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C21" s="22"/>
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C21" s="22" t="n">
+        <x:v>2</x:v>
+      </x:c>
       <x:c r="D21" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Joon</x:v>
       </x:c>
       <x:c r="E21" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>M4 x 8mm stainless bolt &amp; nut set</x:v>
       </x:c>
       <x:c r="F21" s="20" t="str">
-        <x:v>TBD</x:v>
-      </x:c>
-      <x:c r="G21" s="22" t="str">
+        <x:v>https://www.joon.co.za/products/bolt-nut-set</x:v>
+      </x:c>
+      <x:c r="G21" s="22" t="n">
         <x:f>IF(ISNUMBER(C21),B21*C21,"TBD")</x:f>
-        <x:v>TBD</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="H21" s="20" t="str">
-        <x:v>TBD</x:v>
+        <x:v>Candidate</x:v>
       </x:c>
       <x:c r="I21" s="20" t="str">
-        <x:v>Bolts, nuts, washers, standoffs</x:v>
+        <x:v>40 M4 x 8mm stainless bolt-and-nut sets for serviceable panel mounting. Exact lengths may be mixed during fabrication.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1134,7 +1148,7 @@
       <x:c r="F25" s="51"/>
       <x:c r="G25" s="52" t="n">
         <x:f>SUMPRODUCT(B5:B23,C5:C23)</x:f>
-        <x:v>5502.65</x:v>
+        <x:v>8039.15</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1151,14 +1165,14 @@
     <x:row r="28">
       <x:c r="A28" t="n">
         <x:f>COUNT(C5:C22)</x:f>
-        <x:v>10</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B28" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="C28" s="24" t="n">
         <x:f>A28/B28</x:f>
-        <x:v>0.5555555555555556</x:v>
+        <x:v>0.9444444444444444</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="42" customHeight="1">

</xml_diff>

<commit_message>
Update SentinelT BOM project styling
</commit_message>
<xml_diff>
--- a/Documentation/BOM/SentinelT_Bill_of_Materials.xlsx
+++ b/Documentation/BOM/SentinelT_Bill_of_Materials.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="R88e8c55008944177"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Submission_Checklist" sheetId="2" r:id="R4169c6a370e746be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" r:id="Re99f593ceac54329"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Submission_Checklist" sheetId="2" r:id="Reae3f2470bef41af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -480,7 +480,7 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="5" t="str">
-        <x:v>SentinelT Robo Rumble 2026 — Bill of Materials</x:v>
+        <x:v>SentinelT Robo Wars - Bill of Materials</x:v>
       </x:c>
       <x:c r="B1" s="5"/>
       <x:c r="C1" s="5"/>
@@ -502,7 +502,7 @@
         <x:v>Category</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>Robo Wars – RC Combat</x:v>
+        <x:v>Robo Wars - RC Combat</x:v>
       </x:c>
       <x:c r="E2" t="str">
         <x:v>Mass Budget</x:v>
@@ -517,7 +517,7 @@
         <x:v>&lt; 5.000 kg</x:v>
       </x:c>
       <x:c r="I2" t="str">
-        <x:v>NEAR-COMPLETE PROCUREMENT DATA</x:v>
+        <x:v>ENGINEERING PROCUREMENT DATA</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1131,15 +1131,15 @@
         <x:v>TBD</x:v>
       </x:c>
       <x:c r="H24" s="54" t="str">
-        <x:v>Submission Requirement</x:v>
+        <x:v>Project Total</x:v>
       </x:c>
       <x:c r="I24" s="54" t="str">
-        <x:v>Must be fully populated before final submission</x:v>
+        <x:v>Final value becomes numeric when all selected component rows are priced.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="51" t="str">
-        <x:v>VERIFIED CANDIDATE SUBTOTAL (priced rows only)</x:v>
+        <x:v>CURRENT PRICED COMPONENT SUBTOTAL</x:v>
       </x:c>
       <x:c r="B25" s="51"/>
       <x:c r="C25" s="51"/>

</xml_diff>